<commit_message>
Actualización dashboard y diccionario d datos
</commit_message>
<xml_diff>
--- a/extras/diccionario_datos_RetailIQ360.xlsx
+++ b/extras/diccionario_datos_RetailIQ360.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Indice de tablas'!$A$4:$J$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Diccionario completo'!$A$4:$K$229</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Relaciones modelo'!$A$4:$H$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Verificaciones'!$A$4:$E$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Verificaciones'!$A$4:$E$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Orden carga Power BI'!$A$4:$F$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Power BI'!$A$4:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Fuentes no cargar'!$A$4:$F$7</definedName>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Columna region de dim_geografia_ar.</t>
+          <t>Region macro: AMBA, Centro, NOA, NEA, Cuyo, Patagonia.</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Columna provincia de dim_geografia_ar.</t>
+          <t>Nombre completo de la provincia argentina.</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Columna ciudad de dim_geografia_ar.</t>
+          <t>Ciudad o localidad.</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Columna zona de dim_geografia_ar.</t>
+          <t>Zona simplificada: AMBA o Interior.</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Columna peso_facturacion de dim_geografia_ar.</t>
+          <t>Peso relativo de facturacion calibrado con benchmarks CACE (suma 1.0).</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Clave de sucursal; puede estar en blanco en ventas digitales.</t>
+          <t>Clave de sucursal; queda nulo para canales digitales (CanalID 2, 3, 4). No es error.</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Columna nombre de dim_sucursales_ar.</t>
+          <t>Nombre de la sucursal o del cliente (segun la tabla).</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Columna tipo de dim_sucursales_ar.</t>
+          <t>Tipo de sucursal: Tienda grande, Tienda chica, Dark store.</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Columna provincia de dim_sucursales_ar.</t>
+          <t>Nombre completo de la provincia argentina.</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Columna ciudad de dim_sucursales_ar.</t>
+          <t>Ciudad o localidad.</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Columna region de dim_sucursales_ar.</t>
+          <t>Region macro: AMBA, Centro, NOA, NEA, Cuyo, Patagonia.</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Columna m2_ventas de dim_sucursales_ar.</t>
+          <t>Metros cuadrados del area de ventas.</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Columna empleados de dim_sucursales_ar.</t>
+          <t>Cantidad de empleados de la sucursal.</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Columna fecha_apertura de dim_sucursales_ar.</t>
+          <t>Fecha de apertura de la sucursal.</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Columna flag_activa de dim_sucursales_ar.</t>
+          <t>Estado de la sucursal: 1 = activa, 0 = cerrada.</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Columna nombre de dim_canal_ar.</t>
+          <t>Nombre de la sucursal o del cliente (segun la tabla).</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Columna tipo de dim_canal_ar.</t>
+          <t>Tipo de sucursal: Tienda grande, Tienda chica, Dark store.</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Columna plataforma de dim_canal_ar.</t>
+          <t>Plataforma del canal: POS fisico, Sitio web, App iOS/Android, MercadoLibre.</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Columna flag_online de dim_canal_ar.</t>
+          <t>Indicador de canal online: 0 = presencial, 1 = online.</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Columna peso_facturacion de dim_canal_ar.</t>
+          <t>Peso relativo de facturacion calibrado con benchmarks CACE (suma 1.0).</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Columna nombre de dim_clientes_ar.</t>
+          <t>Nombre de la sucursal o del cliente (segun la tabla).</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Columna email de dim_clientes_ar.</t>
+          <t>Correo electronico del cliente (unico en la tabla, generado con Faker).</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>Columna telefono de dim_clientes_ar.</t>
+          <t>Telefono con formato argentino (+54).</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>Columna provincia de dim_clientes_ar.</t>
+          <t>Nombre completo de la provincia argentina.</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>Columna ciudad de dim_clientes_ar.</t>
+          <t>Ciudad o localidad.</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>Columna region de dim_clientes_ar.</t>
+          <t>Region macro: AMBA, Centro, NOA, NEA, Cuyo, Patagonia.</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>Columna zona de dim_clientes_ar.</t>
+          <t>Zona simplificada: AMBA o Interior.</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>Columna nse de dim_clientes_ar.</t>
+          <t>Nivel socioeconomico: ABC1, C2, C3, D (distribucion calibrada con CACE).</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>Columna rango_edad de dim_clientes_ar.</t>
+          <t>Segmento etario: 18-20, 21-29, 30-34, 35-44, 45-59, 60+.</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>Columna genero de dim_clientes_ar.</t>
+          <t>Genero del cliente: M o F (50/50 calibrado con CACE).</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>Columna canal_preferido de dim_clientes_ar.</t>
+          <t>Canal de compra preferido del cliente.</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
@@ -3864,9 +3864,9 @@
           <t>Decimal</t>
         </is>
       </c>
-      <c r="F44" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F44" s="17" t="inlineStr">
+        <is>
+          <t>CALC</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>Columna segmento_rfm de dim_clientes_ar.</t>
+          <t>Columna RFM sin valores en el modelo actual. Eliminar en Power Query (100% nula).</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>Columna fecha_alta de dim_clientes_ar.</t>
+          <t>Fecha de registro del cliente.</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>Variacion mensual del IPC general.</t>
+          <t>Variacion mensual del IPC general (INDEC).</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>Columna ipc_alimentos_bebidas de dim_inflacion_ipc.</t>
+          <t>Variacion mensual del IPC de alimentos y bebidas.</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>Columna ipc_indumentaria_calzado de dim_inflacion_ipc.</t>
+          <t>Variacion mensual del IPC de indumentaria y calzado.</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>Columna ipc_equipamiento_hogar de dim_inflacion_ipc.</t>
+          <t>Variacion mensual del IPC de equipamiento del hogar.</t>
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
-          <t>Columna ipc_transporte de dim_inflacion_ipc.</t>
+          <t>Variacion mensual del IPC de transporte.</t>
         </is>
       </c>
       <c r="J53" s="6" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="I54" s="6" t="inlineStr">
         <is>
-          <t>Columna ipc_comunicacion de dim_inflacion_ipc.</t>
+          <t>Variacion mensual del IPC de comunicacion.</t>
         </is>
       </c>
       <c r="J54" s="6" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="I56" s="6" t="inlineStr">
         <is>
-          <t>Mes numerico del registro.</t>
+          <t>Mes numerico del registro (1 a 12).</t>
         </is>
       </c>
       <c r="J56" s="6" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>Clave mensual numerica: anio * 100 + mes.</t>
+          <t>Clave mensual numerica: anio * 100 + mes (ej: octubre 2017 = 201710).</t>
         </is>
       </c>
       <c r="J57" s="6" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="I58" s="6" t="inlineStr">
         <is>
-          <t>Indice acumulado usado para deflactar precios.</t>
+          <t>Indice acumulado base dic-2016 (= 1.0) usado para deflactar precios.</t>
         </is>
       </c>
       <c r="J58" s="6" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="I61" s="6" t="inlineStr">
         <is>
-          <t>Clave de fecha en formato YYYYMMDD.</t>
+          <t>Clave de fecha en formato YYYYMMDD (ej: 20171015).</t>
         </is>
       </c>
       <c r="J61" s="6" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="I63" s="6" t="inlineStr">
         <is>
-          <t>Columna semestre de dim_tiempo.</t>
+          <t>Semestre del anio (1 o 2).</t>
         </is>
       </c>
       <c r="J63" s="6" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>Trimestre del registro.</t>
+          <t>Trimestre del registro (1 a 4).</t>
         </is>
       </c>
       <c r="J64" s="6" t="inlineStr">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>Mes numerico del registro.</t>
+          <t>Mes numerico del registro (1 a 12).</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>Columna nombre_mes de dim_tiempo.</t>
+          <t>Nombre del mes en espanol (Enero, Febrero... Diciembre).</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>Columna dia de dim_tiempo.</t>
+          <t>Dia del mes (1 a 31).</t>
         </is>
       </c>
       <c r="J67" s="6" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="I68" s="6" t="inlineStr">
         <is>
-          <t>Columna dia_semana de dim_tiempo.</t>
+          <t>Dia de la semana: 0 = lunes, 6 = domingo.</t>
         </is>
       </c>
       <c r="J68" s="6" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="I69" s="6" t="inlineStr">
         <is>
-          <t>Columna nombre_dia de dim_tiempo.</t>
+          <t>Nombre del dia en espanol (Lunes, Martes... Domingo).</t>
         </is>
       </c>
       <c r="J69" s="6" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="I70" s="6" t="inlineStr">
         <is>
-          <t>Columna semana_anio de dim_tiempo.</t>
+          <t>Numero de semana del anio (ISO).</t>
         </is>
       </c>
       <c r="J70" s="6" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>Columna es_fin_semana de dim_tiempo.</t>
+          <t>True para sabado y domingo; False para dias habiles.</t>
         </is>
       </c>
       <c r="J71" s="6" t="inlineStr">
@@ -5308,9 +5308,9 @@
           <t>Texto</t>
         </is>
       </c>
-      <c r="F72" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F72" s="17" t="inlineStr">
+        <is>
+          <t>CALC</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
-          <t>Columna anio_mes de dim_tiempo.</t>
+          <t>Etiqueta YYYY-MM derivada de anio y mes (ej: '2017-10'). Usar para ejes de graficos.</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="I73" s="6" t="inlineStr">
         <is>
-          <t>Clave mensual numerica: anio * 100 + mes.</t>
+          <t>Clave mensual numerica: anio * 100 + mes (ej: octubre 2017 = 201710).</t>
         </is>
       </c>
       <c r="J73" s="6" t="inlineStr">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>Categoria de producto traducida al ingles.</t>
+          <t>Categoria del producto en ingles (72 categorias Olist originales).</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="I78" s="6" t="inlineStr">
         <is>
-          <t>Categoria simplificada en espanol alineada a CACE.</t>
+          <t>Categoria CACE en espanol (10 categorias). FK hacia dim_categorias.</t>
         </is>
       </c>
       <c r="J78" s="6" t="inlineStr">
@@ -5882,7 +5882,7 @@
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>Volumen calculado: largo * alto * ancho.</t>
+          <t>Volumen calculado por el ETL: largo * alto * ancho en cm3.</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>Columna CategoriaID de dim_categorias.</t>
+          <t>Clave primaria de categoria CACE (1 a 10).</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="I86" s="6" t="inlineStr">
         <is>
-          <t>Categoria simplificada en espanol alineada a CACE.</t>
+          <t>Categoria CACE en espanol (10 categorias). FK hacia dim_categorias.</t>
         </is>
       </c>
       <c r="J86" s="6" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="I91" s="9" t="inlineStr">
         <is>
-          <t>Clave de sucursal; puede estar en blanco en ventas digitales.</t>
+          <t>Clave de sucursal; queda nulo para canales digitales (CanalID 2, 3, 4). No es error.</t>
         </is>
       </c>
       <c r="J91" s="9" t="inlineStr">
@@ -6281,7 +6281,7 @@
       </c>
       <c r="I92" s="9" t="inlineStr">
         <is>
-          <t>Clave mensual numerica: anio * 100 + mes.</t>
+          <t>Clave mensual numerica: anio * 100 + mes (ej: octubre 2017 = 201710).</t>
         </is>
       </c>
       <c r="J92" s="9" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="I95" s="9" t="inlineStr">
         <is>
-          <t>Mes numerico del registro.</t>
+          <t>Mes numerico del registro (1 a 12).</t>
         </is>
       </c>
       <c r="J95" s="9" t="inlineStr">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="I96" s="9" t="inlineStr">
         <is>
-          <t>Trimestre del registro.</t>
+          <t>Trimestre del registro (1 a 4).</t>
         </is>
       </c>
       <c r="J96" s="9" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="I97" s="9" t="inlineStr">
         <is>
-          <t>Categoria de producto traducida al ingles.</t>
+          <t>Categoria del producto en ingles (72 categorias Olist originales).</t>
         </is>
       </c>
       <c r="J97" s="9" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="I98" s="9" t="inlineStr">
         <is>
-          <t>Medio de pago asignado con distribucion calibrada por CACE.</t>
+          <t>Medio de pago asignado con distribucion calibrada por CACE 2025.</t>
         </is>
       </c>
       <c r="J98" s="9" t="inlineStr">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="I99" s="9" t="inlineStr">
         <is>
-          <t>Cantidad de cuotas asignada con distribucion calibrada por CACE.</t>
+          <t>Cantidad de cuotas: 1, 3, 6, 10, 15 (distribucion calibrada CACE).</t>
         </is>
       </c>
       <c r="J99" s="9" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="I100" s="9" t="inlineStr">
         <is>
-          <t>Tipo de entrega asignado con benchmarks CACE.</t>
+          <t>Tipo de entrega asignado con benchmarks CACE 2025.</t>
         </is>
       </c>
       <c r="J100" s="9" t="inlineStr">
@@ -6776,7 +6776,7 @@
       </c>
       <c r="I101" s="9" t="inlineStr">
         <is>
-          <t>Plazo de entrega asignado con benchmarks CACE.</t>
+          <t>Plazo de entrega asignado con benchmarks CACE 2024.</t>
         </is>
       </c>
       <c r="J101" s="9" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="I105" s="9" t="inlineStr">
         <is>
-          <t>Tipo de cambio ARS/USD usado como moneda puente.</t>
+          <t>Tipo de cambio ARS/USD del BCRA (forward fill en feriados).</t>
         </is>
       </c>
       <c r="J105" s="9" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="I106" s="9" t="inlineStr">
         <is>
-          <t>Factor BRL a ARS calculado como ars_por_usd / 3.3.</t>
+          <t>Factor de conversion BRL a ARS calculado como ars_por_usd / 3.3.</t>
         </is>
       </c>
       <c r="J106" s="9" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I107" s="9" t="inlineStr">
         <is>
-          <t>Precio nominal en pesos argentinos.</t>
+          <t>Precio nominal en pesos argentinos al tipo de cambio del dia.</t>
         </is>
       </c>
       <c r="J107" s="9" t="inlineStr">
@@ -7161,7 +7161,7 @@
       </c>
       <c r="I108" s="9" t="inlineStr">
         <is>
-          <t>Flete nominal en pesos argentinos.</t>
+          <t>Flete nominal en pesos argentinos al tipo de cambio del dia.</t>
         </is>
       </c>
       <c r="J108" s="9" t="inlineStr">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="I109" s="9" t="inlineStr">
         <is>
-          <t>Variacion mensual del IPC general.</t>
+          <t>Variacion mensual del IPC general (INDEC).</t>
         </is>
       </c>
       <c r="J109" s="9" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="I110" s="9" t="inlineStr">
         <is>
-          <t>Indice acumulado usado para deflactar precios.</t>
+          <t>Indice acumulado base dic-2016 (= 1.0) usado para deflactar precios.</t>
         </is>
       </c>
       <c r="J110" s="9" t="inlineStr">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="I111" s="9" t="inlineStr">
         <is>
-          <t>Precio en pesos argentinos reales, deflactado por IPC.</t>
+          <t>Precio en ARS constantes deflactado a dic-2016 (= precio_venta_ars / indice_ipc_acum).</t>
         </is>
       </c>
       <c r="J111" s="9" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="I112" s="9" t="inlineStr">
         <is>
-          <t>Indica si la fila tiene cobertura de IPC para el periodo.</t>
+          <t>True si la fila tiene cobertura IPC. False solo para sep-dic 2016 (~317 filas).</t>
         </is>
       </c>
       <c r="J112" s="9" t="inlineStr">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="I113" s="9" t="inlineStr">
         <is>
-          <t>Identificador original de orden Olist.</t>
+          <t>Identificador original de orden Olist (trazabilidad).</t>
         </is>
       </c>
       <c r="J113" s="9" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="I115" s="9" t="inlineStr">
         <is>
-          <t>Identificador original del vendedor Olist.</t>
+          <t>Identificador original del vendedor Olist (trazabilidad).</t>
         </is>
       </c>
       <c r="J115" s="9" t="inlineStr">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="I117" s="9" t="inlineStr">
         <is>
-          <t>Clave del registro de precio de competencia.</t>
+          <t>Clave primaria del registro de precio de competencia.</t>
         </is>
       </c>
       <c r="J117" s="9" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="I120" s="9" t="inlineStr">
         <is>
-          <t>Mes numerico del registro.</t>
+          <t>Mes numerico del registro (1 a 12).</t>
         </is>
       </c>
       <c r="J120" s="9" t="inlineStr">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="I121" s="9" t="inlineStr">
         <is>
-          <t>Fecha del relevamiento de precios.</t>
+          <t>Dia 15 de cada mes. FK hacia dim_tiempo.fecha (relacion manual en Power BI).</t>
         </is>
       </c>
       <c r="J121" s="9" t="inlineStr">
@@ -7938,7 +7938,7 @@
       </c>
       <c r="I123" s="9" t="inlineStr">
         <is>
-          <t>Precio online propio en ARS.</t>
+          <t>Precio online propio en ARS (menor que precio_lista_ars en la mayoria de los casos).</t>
         </is>
       </c>
       <c r="J123" s="9" t="inlineStr">
@@ -8048,7 +8048,7 @@
       </c>
       <c r="I125" s="9" t="inlineStr">
         <is>
-          <t>Porcentaje de descuento aplicado.</t>
+          <t>Porcentaje de descuento aplicado (entre 0 y 1).</t>
         </is>
       </c>
       <c r="J125" s="9" t="inlineStr">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="I126" s="9" t="inlineStr">
         <is>
-          <t>Indice precio propio / precio competencia.</t>
+          <t>Indice precio propio / precio competencia. Menor que 1 = precio propio mas barato.</t>
         </is>
       </c>
       <c r="J126" s="9" t="inlineStr">
@@ -8213,7 +8213,7 @@
       </c>
       <c r="I128" s="9" t="inlineStr">
         <is>
-          <t>Clave mensual numerica: anio * 100 + mes.</t>
+          <t>Clave mensual numerica: anio * 100 + mes (ej: octubre 2017 = 201710).</t>
         </is>
       </c>
       <c r="J128" s="9" t="inlineStr">
@@ -10400,7 +10400,7 @@
       </c>
       <c r="I173" s="12" t="inlineStr">
         <is>
-          <t>Medio de pago asignado con distribucion calibrada por CACE.</t>
+          <t>Medio de pago asignado con distribucion calibrada por CACE 2025.</t>
         </is>
       </c>
       <c r="J173" s="12" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="I174" s="12" t="inlineStr">
         <is>
-          <t>Columna tipo de cace_04a_medios_pago_oferta.</t>
+          <t>Tipo de sucursal: Tienda grande, Tienda chica, Dark store.</t>
         </is>
       </c>
       <c r="J174" s="12" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="I191" s="12" t="inlineStr">
         <is>
-          <t>Tipo de entrega asignado con benchmarks CACE.</t>
+          <t>Tipo de entrega asignado con benchmarks CACE 2025.</t>
         </is>
       </c>
       <c r="J191" s="12" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="I199" s="12" t="inlineStr">
         <is>
-          <t>Plazo de entrega asignado con benchmarks CACE.</t>
+          <t>Plazo de entrega asignado con benchmarks CACE 2024.</t>
         </is>
       </c>
       <c r="J199" s="12" t="inlineStr">
@@ -12188,7 +12188,7 @@
       </c>
       <c r="I209" s="12" t="inlineStr">
         <is>
-          <t>Columna region de cace_06a_distribucion_regional.</t>
+          <t>Region macro: AMBA, Centro, NOA, NEA, Cuyo, Patagonia.</t>
         </is>
       </c>
       <c r="J209" s="12" t="inlineStr">
@@ -13857,7 +13857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13909,63 +13909,63 @@
       </c>
       <c r="B4" s="28" t="inlineStr">
         <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Desactivar Fecha/hora automatica antes de cargar: Archivo &gt; Opciones &gt; Archivo actual &gt; Carga de datos.</t>
+        </is>
+      </c>
+      <c r="E4" s="29" t="inlineStr"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>Configurar regional del archivo como Ingles (EE.UU.) al importar CSV: separador decimal = punto.</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
           <t>dim_tiempo</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>Formato</t>
         </is>
       </c>
-      <c r="D4" s="28" t="inlineStr">
-        <is>
-          <t>Marcar como tabla de fechas usando dim_tiempo[fecha].</t>
-        </is>
-      </c>
-      <c r="E4" s="29" t="inlineStr"/>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="inlineStr">
-        <is>
-          <t>dim_tiempo</t>
-        </is>
-      </c>
-      <c r="C5" s="30" t="inlineStr">
-        <is>
-          <t>Integridad</t>
-        </is>
-      </c>
-      <c r="D5" s="31" t="inlineStr">
-        <is>
-          <t>Debe cubrir 2016-01-01 a 2024-12-31 para ventas y precios de competencia.</t>
-        </is>
-      </c>
-      <c r="E5" s="29" t="inlineStr"/>
-    </row>
-    <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B6" s="31" t="inlineStr">
-        <is>
-          <t>dim_clientes_ar</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>Integridad</t>
-        </is>
-      </c>
-      <c r="D6" s="31" t="inlineStr">
-        <is>
-          <t>ClienteID debe ser unico y todos los ClienteID de fact_ventas_final deben existir.</t>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Marcar como Date Table: seleccionar tabla &gt; Herramientas de tabla &gt; Marcar como tabla de fechas &gt; columna fecha.</t>
         </is>
       </c>
       <c r="E6" s="29" t="inlineStr"/>
@@ -13978,7 +13978,7 @@
       </c>
       <c r="B7" s="31" t="inlineStr">
         <is>
-          <t>dim_clientes_ar</t>
+          <t>dim_tiempo</t>
         </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
@@ -13988,7 +13988,7 @@
       </c>
       <c r="D7" s="31" t="inlineStr">
         <is>
-          <t>GeografiaID no debe tener nulos.</t>
+          <t>3.288 filas exactas. Cubre 2016-01-01 a 2024-12-31 incluyendo bisiestos 2016, 2020 y 2024.</t>
         </is>
       </c>
       <c r="E7" s="29" t="inlineStr"/>
@@ -14001,7 +14001,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>dim_inflacion_ipc</t>
+          <t>dim_tiempo</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
@@ -14011,7 +14011,7 @@
       </c>
       <c r="D8" s="31" t="inlineStr">
         <is>
-          <t>PeriodoID debe ser unico y cubrir los PeriodoID usados por fact_ventas_final y fact_precios_comp.</t>
+          <t>La columna fecha cubre todos los valores de fact_ventas_final.fecha y fact_precios_comp.fecha_relevamiento.</t>
         </is>
       </c>
       <c r="E8" s="29" t="inlineStr"/>
@@ -14024,7 +14024,7 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>dim_productos</t>
+          <t>dim_clientes_ar</t>
         </is>
       </c>
       <c r="C9" s="30" t="inlineStr">
@@ -14034,53 +14034,53 @@
       </c>
       <c r="D9" s="31" t="inlineStr">
         <is>
-          <t>product_id debe ser unico y cubrir todos los product_id de fact_ventas_final.</t>
+          <t>10.000 filas exactas. ClienteID unico y todos los ClienteID de fact_ventas_final deben existir.</t>
         </is>
       </c>
       <c r="E9" s="29" t="inlineStr"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>dim_productos</t>
-        </is>
-      </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>dim_clientes_ar</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>Integridad</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr">
+        <is>
+          <t>GeografiaID sin nulos (el ETL aplica fallback por provincia).</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>dim_clientes_ar</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
         <is>
           <t>Negocio</t>
         </is>
       </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>categoria_es debe tener categorias CACE consistentes para vincular con fact_precios_comp.</t>
-        </is>
-      </c>
-      <c r="E10" s="29" t="inlineStr"/>
-    </row>
-    <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="inlineStr">
-        <is>
-          <t>dim_categorias</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>Integridad</t>
-        </is>
-      </c>
-      <c r="D11" s="31" t="inlineStr">
-        <is>
-          <t>categoria_es debe ser unico; es la tabla puente entre productos y precios.</t>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>Eliminar columna segmento_rfm en Power Query: es 100% nula y no aporta al modelo.</t>
         </is>
       </c>
       <c r="E11" s="29" t="inlineStr"/>
@@ -14093,7 +14093,7 @@
       </c>
       <c r="B12" s="31" t="inlineStr">
         <is>
-          <t>fact_ventas_final</t>
+          <t>dim_inflacion_ipc</t>
         </is>
       </c>
       <c r="C12" s="30" t="inlineStr">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="D12" s="31" t="inlineStr">
         <is>
-          <t>Debe tener 110.197 filas y 28 columnas.</t>
+          <t>PeriodoID unico y continuo. Debe cubrir todos los PeriodoID de fact_ventas_final y fact_precios_comp.</t>
         </is>
       </c>
       <c r="E12" s="29" t="inlineStr"/>
@@ -14116,7 +14116,7 @@
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>fact_ventas_final</t>
+          <t>dim_inflacion_ipc</t>
         </is>
       </c>
       <c r="C13" s="32" t="inlineStr">
@@ -14126,30 +14126,30 @@
       </c>
       <c r="D13" s="33" t="inlineStr">
         <is>
-          <t>precio_venta_ars y precio_venta_ars_real deben ser positivos.</t>
+          <t>indice_ipc_acum empieza en 1.0 (dic-2016) y es siempre creciente.</t>
         </is>
       </c>
       <c r="E13" s="29" t="inlineStr"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>fact_ventas_final</t>
-        </is>
-      </c>
-      <c r="C14" s="32" t="inlineStr">
-        <is>
-          <t>Negocio</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>SucursalID puede estar en blanco para canales digitales; no corregirlo como error.</t>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>dim_productos</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Integridad</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
+          <t>32.951 filas exactas. product_id unico y cubre todos los product_id de fact_ventas_final.</t>
         </is>
       </c>
       <c r="E14" s="29" t="inlineStr"/>
@@ -14162,7 +14162,7 @@
       </c>
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>fact_precios_comp</t>
+          <t>dim_productos</t>
         </is>
       </c>
       <c r="C15" s="30" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="D15" s="31" t="inlineStr">
         <is>
-          <t>Debe tener PeriodoID y 360 filas procesadas.</t>
+          <t>Sin nulos en dimensiones fisicas (product_weight_g, length, height, width). Imputadas con mediana.</t>
         </is>
       </c>
       <c r="E15" s="29" t="inlineStr"/>
@@ -14185,69 +14185,391 @@
       </c>
       <c r="B16" s="33" t="inlineStr">
         <is>
+          <t>dim_productos</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="inlineStr">
+        <is>
+          <t>Negocio</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>categoria_es tiene exactamente 10 valores distintos (las 10 categorias CACE).</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="inlineStr"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>dim_categorias</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>Integridad</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>10 filas exactas. Los 10 valores de categoria_es coinciden exactamente en dim_productos y fact_precios_comp.</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="inlineStr"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="inlineStr">
+        <is>
+          <t>fact_ventas_final</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Integridad</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>110.197 filas exactas y 28 columnas. VentaID unico.</t>
+        </is>
+      </c>
+      <c r="E18" s="29" t="inlineStr"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>fact_ventas_final</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>Integridad</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>fecha entre 2016-09-02 y 2018-08-29.</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="inlineStr"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>fact_ventas_final</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>Negocio</t>
+        </is>
+      </c>
+      <c r="D20" s="33" t="inlineStr">
+        <is>
+          <t>precio_venta_ars y precio_venta_ars_real positivos (sin ceros ni negativos).</t>
+        </is>
+      </c>
+      <c r="E20" s="29" t="inlineStr"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B21" s="33" t="inlineStr">
+        <is>
+          <t>fact_ventas_final</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>Negocio</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>SucursalID es nulo para CanalID 2, 3 y 4 (~92% de las filas). No corregir como error.</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr"/>
+    </row>
+    <row r="22" ht="25" customHeight="1">
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>fact_ventas_final</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>Negocio</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="inlineStr">
+        <is>
+          <t>tiene_ipc es False solo para ventas de sep-dic 2016 (~317 filas). indice_ipc_acum = 1.0 en esas filas.</t>
+        </is>
+      </c>
+      <c r="E22" s="29" t="inlineStr"/>
+    </row>
+    <row r="23" ht="25" customHeight="1">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t>fact_ventas_final</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Negocio</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="inlineStr">
+        <is>
+          <t>precio_venta_ars_real es siempre menor o igual a precio_venta_ars (el deflactor nunca infla el precio).</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr"/>
+    </row>
+    <row r="24" ht="25" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
           <t>fact_precios_comp</t>
         </is>
       </c>
-      <c r="C16" s="32" t="inlineStr">
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>Integridad</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="inlineStr">
+        <is>
+          <t>360 filas exactas: 10 categorias x 12 meses x 3 anios (2022-2024).</t>
+        </is>
+      </c>
+      <c r="E24" s="29" t="inlineStr"/>
+    </row>
+    <row r="25" ht="25" customHeight="1">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>fact_precios_comp</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
         <is>
           <t>Negocio</t>
         </is>
       </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>price_index menor que 1 indica precio propio mas barato que competencia.</t>
-        </is>
-      </c>
-      <c r="E16" s="29" t="inlineStr"/>
-    </row>
-    <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>fecha_relevamiento es siempre el dia 15 del mes. Verificar que exista en dim_tiempo.fecha.</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr"/>
+    </row>
+    <row r="26" ht="25" customHeight="1">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>fact_precios_comp</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>Negocio</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>descuento_pct entre 0 y 1. price_index positivo. precio_web_ars &lt; precio_lista_ars en la mayoria.</t>
+        </is>
+      </c>
+      <c r="E26" s="29" t="inlineStr"/>
+    </row>
+    <row r="27" ht="25" customHeight="1">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B27" s="33" t="inlineStr">
+        <is>
+          <t>fact_precios_comp</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>Negocio</t>
+        </is>
+      </c>
+      <c r="D27" s="33" t="inlineStr">
+        <is>
+          <t>price_index &lt; 1 indica precio propio mas barato que competencia.</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="inlineStr"/>
+    </row>
+    <row r="28" ht="25" customHeight="1">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>Crear manualmente: fact_precios_comp[fecha_relevamiento] &gt; dim_tiempo[fecha] (columnas con nombres distintos).</t>
+        </is>
+      </c>
+      <c r="E28" s="29" t="inlineStr"/>
+    </row>
+    <row r="29" ht="25" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>Crear manualmente: fact_precios_comp[categoria] &gt; dim_categorias[categoria_es] (columnas con nombres distintos).</t>
+        </is>
+      </c>
+      <c r="E29" s="29" t="inlineStr"/>
+    </row>
+    <row r="30" ht="25" customHeight="1">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>Eliminar relaciones automaticas incorrectas, especialmente por category_en u otras columnas de texto.</t>
+        </is>
+      </c>
+      <c r="E30" s="29" t="inlineStr"/>
+    </row>
+    <row r="31" ht="25" customHeight="1">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>Verificar que fact_ventas_final &gt; dim_productos use product_id, no category_en.</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="inlineStr"/>
+    </row>
+    <row r="32" ht="25" customHeight="1">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>Benchmarks CACE</t>
         </is>
       </c>
-      <c r="C17" s="22" t="inlineStr">
+      <c r="C32" s="22" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr">
-        <is>
-          <t>No crear relaciones formales automaticas con tablas CACE salvo decision explicita de visualizacion.</t>
-        </is>
-      </c>
-      <c r="E17" s="29" t="inlineStr"/>
-    </row>
-    <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="22" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>Power BI</t>
-        </is>
-      </c>
-      <c r="C18" s="22" t="inlineStr">
-        <is>
-          <t>Modelo</t>
-        </is>
-      </c>
-      <c r="D18" s="24" t="inlineStr">
-        <is>
-          <t>Eliminar relaciones automaticas incorrectas, especialmente por category_en o columnas de texto similares.</t>
-        </is>
-      </c>
-      <c r="E18" s="29" t="inlineStr"/>
+      <c r="D32" s="24" t="inlineStr">
+        <is>
+          <t>No crear relaciones formales con tablas CACE. Usarlas directamente en visualizaciones de comparacion.</t>
+        </is>
+      </c>
+      <c r="E32" s="29" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E18"/>
+  <autoFilter ref="A4:E32"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -15053,7 +15375,7 @@
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>2026-05-25 17:55</t>
+          <t>2026-05-25 18:07</t>
         </is>
       </c>
       <c r="E5" s="38" t="inlineStr">

</xml_diff>